<commit_message>
menu: Τρίτη 21/7 + add 8 new dishes with placeholder prices
Fix tab-name matching bug for "Αναψυκτικά / Ποτά" (xlsx tab uses a
dash, menu-today.txt uses a slash) introduced by the previous merge.

New dishes (prices are placeholders, pending the owner's real board
prices): Ψαρόσουπα, Γεμιστά με κιμά, Μπάμιες με μπούτια, Κεφτεδάκια
τηγανητά/κοκκινιστά, Πένες με κιμά/αλά κρεμ, Φιλετάκια κοτόπουλο αλά κρεμ.
</commit_message>
<xml_diff>
--- a/DAILY_MENU.xlsx
+++ b/DAILY_MENU.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Μαγειρευτά" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Της ώρας" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Συνοδευτικά" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Σαλάτες" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Γλυκά" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Αναψυκτικά - Ποτά" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Μαγειρευτά" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Της ώρας" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Συνοδευτικά" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Σαλάτες" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Γλυκά" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Αναψυκτικά - Ποτά" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,7 +76,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -88,6 +88,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -453,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -814,6 +815,84 @@
       </c>
       <c r="C27" s="4" t="n">
         <v>9.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Ψαρόσουπα</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Γεμιστά με κιμά</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Μπάμιες με μπούτια</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Κεφτεδάκια κοκκινιστά</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Πένες με κιμά</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Πένες αλά κρεμ</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -827,7 +906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1045,6 +1124,32 @@
       </c>
       <c r="C16" s="4" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Κεφτεδάκια τηγανητά</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>7.5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Φιλετάκια κοτόπουλο αλά κρεμ</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>9.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>